<commit_message>
v2 products after competitive research: deeper features + real listing screenshots
Budget template gains Year Overview (12-month trend + category heatmap),
Savings Goals (months-left / monthly-needed math), and a Bills tab.
Invoice tracker gains quarterly summary, avg days-to-pay, collection
rate, avg invoice, and overdue KPIs. Bookkeeping tracker gains quarterly
P&L and per-platform fees paid / fee %. All 37 dashboard values verified
against hand-computed totals; zero formula errors on recalculation.

Listings get keyword-front-loaded titles and galleries of real, unedited
screenshots exported from the actual workbooks (listings/screenshots/).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014AkUe8kkZr9XS2EdNVryQd
</commit_message>
<xml_diff>
--- a/products/freelance-invoice-income-tracker.xlsx
+++ b/products/freelance-invoice-income-tracker.xlsx
@@ -15,7 +15,11 @@
     <sheet name="Dashboard" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
+    <definedName function="false" hidden="false" localSheetId="4" name="_xlnm.Print_Area" vbProcedure="false">Dashboard!$A$1:$M$52</definedName>
+    <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Area" vbProcedure="false">'Income Log'!$A$1:$G$40</definedName>
     <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Area" vbProcedure="false">Invoice!$A$1:$D$35</definedName>
+    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">Settings!$A$1:$D$38</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">'Start Here'!$A$1:$H$26</definedName>
     <definedName function="false" hidden="false" name="ClientList" vbProcedure="false">Settings!$A$18:$A$37</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -28,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="110">
   <si>
     <t xml:space="preserve">Freelance Invoice + Income Tracker</t>
   </si>
@@ -276,6 +280,18 @@
     <t xml:space="preserve">INVOICES SENT</t>
   </si>
   <si>
+    <t xml:space="preserve">AVG DAYS TO PAY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COLLECTION RATE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AVG INVOICE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OVERDUE AMOUNT</t>
+  </si>
+  <si>
     <t xml:space="preserve">Invoiced by month</t>
   </si>
   <si>
@@ -325,20 +341,42 @@
   </si>
   <si>
     <t xml:space="preserve">December</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quarter by quarter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quarter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Collected</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q4</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="mm/dd/yyyy"/>
     <numFmt numFmtId="167" formatCode="\$#,##0.00"/>
     <numFmt numFmtId="168" formatCode="\$#,##0"/>
     <numFmt numFmtId="169" formatCode="0"/>
-    <numFmt numFmtId="170" formatCode="\$#,##0;&quot;($&quot;#,##0\);\-"/>
+    <numFmt numFmtId="170" formatCode="0.0"/>
+    <numFmt numFmtId="171" formatCode="\$#,##0;&quot;($&quot;#,##0\);\-"/>
   </numFmts>
   <fonts count="27">
     <font>
@@ -660,7 +698,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="51">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -833,6 +871,18 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="170" fontId="23" fillId="4" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="21" fillId="4" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="23" fillId="4" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -841,7 +891,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="171" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -849,7 +899,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="171" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1022,7 +1072,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Dashboard!C11</c:f>
+              <c:f>Dashboard!C14</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1067,7 +1117,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Dashboard!$B$12:$B$23</c:f>
+              <c:f>Dashboard!$B$15:$B$26</c:f>
               <c:strCache>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
@@ -1111,7 +1161,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Dashboard!$C$12:$C$23</c:f>
+              <c:f>Dashboard!$C$15:$C$26</c:f>
               <c:numCache>
                 <c:formatCode>\$#,##0;"($"#,##0\);\-</c:formatCode>
                 <c:ptCount val="12"/>
@@ -1157,11 +1207,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="25708349"/>
-        <c:axId val="34290226"/>
+        <c:axId val="94434206"/>
+        <c:axId val="95124837"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="25708349"/>
+        <c:axId val="94434206"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1193,7 +1243,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="34290226"/>
+        <c:crossAx val="95124837"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1201,7 +1251,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="34290226"/>
+        <c:axId val="95124837"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1243,7 +1293,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="25708349"/>
+        <c:crossAx val="94434206"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1275,15 +1325,15 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>4</xdr:col>
+      <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>25</xdr:row>
+      <xdr:row>35</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>65520</xdr:colOff>
-      <xdr:row>40</xdr:row>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>1132560</xdr:colOff>
+      <xdr:row>50</xdr:row>
       <xdr:rowOff>93960</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
@@ -1292,7 +1342,7 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="3378240" y="5133960"/>
+        <a:off x="355680" y="7153200"/>
         <a:ext cx="5399640" cy="2951640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -1485,7 +1535,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <tabColor rgb="FF2E9E8F"/>
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:H25"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -1642,8 +1692,8 @@
     <mergeCell ref="C18:H18"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -1655,7 +1705,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <tabColor rgb="FF1F3A5F"/>
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:H37"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -1909,8 +1959,8 @@
     <mergeCell ref="A2:H2"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -2221,7 +2271,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <tabColor rgb="FF1F3A5F"/>
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:H105"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -3255,8 +3305,8 @@
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -3268,9 +3318,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <tabColor rgb="FF2E9E8F"/>
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:L31"/>
+  <dimension ref="A1:L34"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
@@ -3364,353 +3414,465 @@
       </c>
       <c r="L7" s="42"/>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="5" t="s">
+    <row r="8" customFormat="false" ht="6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B9" s="38" t="s">
         <v>82</v>
       </c>
-      <c r="H10" s="5" t="s">
+      <c r="C9" s="38"/>
+      <c r="E9" s="38" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="15" t="s">
+      <c r="F9" s="38"/>
+      <c r="H9" s="38" t="s">
         <v>84</v>
       </c>
-      <c r="B11" s="15" t="s">
+      <c r="I9" s="38"/>
+      <c r="K9" s="38" t="s">
         <v>85</v>
       </c>
-      <c r="C11" s="15" t="s">
+      <c r="L9" s="38"/>
+    </row>
+    <row r="10" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B10" s="43" t="n">
+        <f aca="false">IFERROR(ROUND(SUMPRODUCT(('Income Log'!$G$6:$G$105-'Income Log'!$A$6:$A$105)*('Income Log'!$G$6:$G$105&lt;&gt;"")*(YEAR('Income Log'!$A$6:$A$105)=$C$4))/SUMPRODUCT(('Income Log'!$G$6:$G$105&lt;&gt;"")*(YEAR('Income Log'!$A$6:$A$105)=$C$4)*1),1),"—")</f>
+        <v>10</v>
+      </c>
+      <c r="C10" s="43"/>
+      <c r="E10" s="44" t="n">
+        <f aca="false">IF(B7=0,"",E7/B7)</f>
+        <v>0.797979797979798</v>
+      </c>
+      <c r="F10" s="44"/>
+      <c r="H10" s="45" t="n">
+        <f aca="false">IF(K7=0,"",B7/K7)</f>
+        <v>990</v>
+      </c>
+      <c r="I10" s="45"/>
+      <c r="K10" s="41" t="n">
+        <f aca="false">SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$F$6:$F$105,"Overdue",'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,1,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4+1,1,1))</f>
+        <v>0</v>
+      </c>
+      <c r="L10" s="41"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="H11" s="15" t="s">
+      <c r="H13" s="5" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="B14" s="15" t="s">
+        <v>89</v>
+      </c>
+      <c r="C14" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="H14" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="I11" s="15" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="43" t="n">
+      <c r="I14" s="15" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="46" t="n">
         <v>1</v>
       </c>
-      <c r="B12" s="44" t="s">
-        <v>87</v>
-      </c>
-      <c r="C12" s="45" t="n">
-        <f aca="false">SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,$A12,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4,$A12+1,1))</f>
+      <c r="B15" s="47" t="s">
+        <v>91</v>
+      </c>
+      <c r="C15" s="48" t="n">
+        <f aca="false">SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,$A15,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4,$A15+1,1))</f>
         <v>1520</v>
       </c>
-      <c r="H12" s="44" t="str">
+      <c r="H15" s="47" t="str">
         <f aca="false">IF(Settings!A18="","",Settings!A18)</f>
         <v>Acme Studios</v>
       </c>
-      <c r="I12" s="45" t="n">
-        <f aca="false">IF($H12="","",SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$B$6:$B$105,$H12,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,1,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4+1,1,1)))</f>
+      <c r="I15" s="48" t="n">
+        <f aca="false">IF($H15="","",SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$B$6:$B$105,$H15,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,1,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4+1,1,1)))</f>
         <v>2120</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="43" t="n">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="46" t="n">
         <v>2</v>
       </c>
-      <c r="B13" s="44" t="s">
-        <v>88</v>
-      </c>
-      <c r="C13" s="45" t="n">
-        <f aca="false">SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,$A13,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4,$A13+1,1))</f>
+      <c r="B16" s="47" t="s">
+        <v>92</v>
+      </c>
+      <c r="C16" s="48" t="n">
+        <f aca="false">SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,$A16,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4,$A16+1,1))</f>
         <v>850</v>
       </c>
-      <c r="H13" s="44" t="str">
+      <c r="H16" s="47" t="str">
         <f aca="false">IF(Settings!A19="","",Settings!A19)</f>
         <v>Beacon Coffee Co.</v>
       </c>
-      <c r="I13" s="45" t="n">
-        <f aca="false">IF($H13="","",SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$B$6:$B$105,$H13,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,1,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4+1,1,1)))</f>
+      <c r="I16" s="48" t="n">
+        <f aca="false">IF($H16="","",SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$B$6:$B$105,$H16,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,1,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4+1,1,1)))</f>
         <v>850</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="43" t="n">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="B14" s="44" t="s">
-        <v>89</v>
-      </c>
-      <c r="C14" s="45" t="n">
-        <f aca="false">SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,$A14,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4,$A14+1,1))</f>
+      <c r="B17" s="47" t="s">
+        <v>93</v>
+      </c>
+      <c r="C17" s="48" t="n">
+        <f aca="false">SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,$A17,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4,$A17+1,1))</f>
         <v>600</v>
       </c>
-      <c r="H14" s="44" t="str">
+      <c r="H17" s="47" t="str">
         <f aca="false">IF(Settings!A20="","",Settings!A20)</f>
         <v/>
       </c>
-      <c r="I14" s="45" t="str">
-        <f aca="false">IF($H14="","",SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$B$6:$B$105,$H14,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,1,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4+1,1,1)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="43" t="n">
+      <c r="I17" s="48" t="str">
+        <f aca="false">IF($H17="","",SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$B$6:$B$105,$H17,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,1,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4+1,1,1)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="46" t="n">
         <v>4</v>
       </c>
-      <c r="B15" s="44" t="s">
-        <v>90</v>
-      </c>
-      <c r="C15" s="45" t="n">
-        <f aca="false">SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,$A15,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4,$A15+1,1))</f>
-        <v>0</v>
-      </c>
-      <c r="H15" s="44" t="str">
-        <f aca="false">IF(Settings!A21="","",Settings!A21)</f>
-        <v/>
-      </c>
-      <c r="I15" s="45" t="str">
-        <f aca="false">IF($H15="","",SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$B$6:$B$105,$H15,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,1,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4+1,1,1)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="43" t="n">
-        <v>5</v>
-      </c>
-      <c r="B16" s="44" t="s">
-        <v>91</v>
-      </c>
-      <c r="C16" s="45" t="n">
-        <f aca="false">SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,$A16,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4,$A16+1,1))</f>
-        <v>0</v>
-      </c>
-      <c r="H16" s="44" t="str">
-        <f aca="false">IF(Settings!A22="","",Settings!A22)</f>
-        <v/>
-      </c>
-      <c r="I16" s="45" t="str">
-        <f aca="false">IF($H16="","",SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$B$6:$B$105,$H16,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,1,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4+1,1,1)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="43" t="n">
-        <v>6</v>
-      </c>
-      <c r="B17" s="44" t="s">
-        <v>92</v>
-      </c>
-      <c r="C17" s="45" t="n">
-        <f aca="false">SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,$A17,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4,$A17+1,1))</f>
-        <v>0</v>
-      </c>
-      <c r="H17" s="44" t="str">
-        <f aca="false">IF(Settings!A23="","",Settings!A23)</f>
-        <v/>
-      </c>
-      <c r="I17" s="45" t="str">
-        <f aca="false">IF($H17="","",SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$B$6:$B$105,$H17,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,1,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4+1,1,1)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="43" t="n">
-        <v>7</v>
-      </c>
-      <c r="B18" s="44" t="s">
-        <v>93</v>
-      </c>
-      <c r="C18" s="45" t="n">
+      <c r="B18" s="47" t="s">
+        <v>94</v>
+      </c>
+      <c r="C18" s="48" t="n">
         <f aca="false">SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,$A18,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4,$A18+1,1))</f>
         <v>0</v>
       </c>
-      <c r="H18" s="44" t="str">
-        <f aca="false">IF(Settings!A24="","",Settings!A24)</f>
-        <v/>
-      </c>
-      <c r="I18" s="45" t="str">
+      <c r="H18" s="47" t="str">
+        <f aca="false">IF(Settings!A21="","",Settings!A21)</f>
+        <v/>
+      </c>
+      <c r="I18" s="48" t="str">
         <f aca="false">IF($H18="","",SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$B$6:$B$105,$H18,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,1,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4+1,1,1)))</f>
         <v/>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="43" t="n">
-        <v>8</v>
-      </c>
-      <c r="B19" s="44" t="s">
-        <v>94</v>
-      </c>
-      <c r="C19" s="45" t="n">
+      <c r="A19" s="46" t="n">
+        <v>5</v>
+      </c>
+      <c r="B19" s="47" t="s">
+        <v>95</v>
+      </c>
+      <c r="C19" s="48" t="n">
         <f aca="false">SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,$A19,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4,$A19+1,1))</f>
         <v>0</v>
       </c>
-      <c r="H19" s="44" t="str">
-        <f aca="false">IF(Settings!A25="","",Settings!A25)</f>
-        <v/>
-      </c>
-      <c r="I19" s="45" t="str">
+      <c r="H19" s="47" t="str">
+        <f aca="false">IF(Settings!A22="","",Settings!A22)</f>
+        <v/>
+      </c>
+      <c r="I19" s="48" t="str">
         <f aca="false">IF($H19="","",SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$B$6:$B$105,$H19,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,1,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4+1,1,1)))</f>
         <v/>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="43" t="n">
-        <v>9</v>
-      </c>
-      <c r="B20" s="44" t="s">
-        <v>95</v>
-      </c>
-      <c r="C20" s="45" t="n">
+      <c r="A20" s="46" t="n">
+        <v>6</v>
+      </c>
+      <c r="B20" s="47" t="s">
+        <v>96</v>
+      </c>
+      <c r="C20" s="48" t="n">
         <f aca="false">SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,$A20,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4,$A20+1,1))</f>
         <v>0</v>
       </c>
-      <c r="H20" s="44" t="str">
-        <f aca="false">IF(Settings!A26="","",Settings!A26)</f>
-        <v/>
-      </c>
-      <c r="I20" s="45" t="str">
+      <c r="H20" s="47" t="str">
+        <f aca="false">IF(Settings!A23="","",Settings!A23)</f>
+        <v/>
+      </c>
+      <c r="I20" s="48" t="str">
         <f aca="false">IF($H20="","",SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$B$6:$B$105,$H20,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,1,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4+1,1,1)))</f>
         <v/>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="43" t="n">
-        <v>10</v>
-      </c>
-      <c r="B21" s="44" t="s">
-        <v>96</v>
-      </c>
-      <c r="C21" s="45" t="n">
+      <c r="A21" s="46" t="n">
+        <v>7</v>
+      </c>
+      <c r="B21" s="47" t="s">
+        <v>97</v>
+      </c>
+      <c r="C21" s="48" t="n">
         <f aca="false">SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,$A21,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4,$A21+1,1))</f>
         <v>0</v>
       </c>
-      <c r="H21" s="44" t="str">
-        <f aca="false">IF(Settings!A27="","",Settings!A27)</f>
-        <v/>
-      </c>
-      <c r="I21" s="45" t="str">
+      <c r="H21" s="47" t="str">
+        <f aca="false">IF(Settings!A24="","",Settings!A24)</f>
+        <v/>
+      </c>
+      <c r="I21" s="48" t="str">
         <f aca="false">IF($H21="","",SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$B$6:$B$105,$H21,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,1,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4+1,1,1)))</f>
         <v/>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="43" t="n">
-        <v>11</v>
-      </c>
-      <c r="B22" s="44" t="s">
-        <v>97</v>
-      </c>
-      <c r="C22" s="45" t="n">
+      <c r="A22" s="46" t="n">
+        <v>8</v>
+      </c>
+      <c r="B22" s="47" t="s">
+        <v>98</v>
+      </c>
+      <c r="C22" s="48" t="n">
         <f aca="false">SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,$A22,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4,$A22+1,1))</f>
         <v>0</v>
       </c>
-      <c r="H22" s="46" t="str">
-        <f aca="false">IF(Settings!A28="","",Settings!A28)</f>
-        <v/>
-      </c>
-      <c r="I22" s="47" t="str">
+      <c r="H22" s="47" t="str">
+        <f aca="false">IF(Settings!A25="","",Settings!A25)</f>
+        <v/>
+      </c>
+      <c r="I22" s="48" t="str">
         <f aca="false">IF($H22="","",SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$B$6:$B$105,$H22,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,1,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4+1,1,1)))</f>
         <v/>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="43" t="n">
-        <v>12</v>
-      </c>
-      <c r="B23" s="44" t="s">
-        <v>98</v>
-      </c>
-      <c r="C23" s="45" t="n">
+      <c r="A23" s="46" t="n">
+        <v>9</v>
+      </c>
+      <c r="B23" s="47" t="s">
+        <v>99</v>
+      </c>
+      <c r="C23" s="48" t="n">
         <f aca="false">SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,$A23,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4,$A23+1,1))</f>
         <v>0</v>
       </c>
-      <c r="H23" s="46" t="str">
+      <c r="H23" s="47" t="str">
+        <f aca="false">IF(Settings!A26="","",Settings!A26)</f>
+        <v/>
+      </c>
+      <c r="I23" s="48" t="str">
+        <f aca="false">IF($H23="","",SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$B$6:$B$105,$H23,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,1,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4+1,1,1)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="46" t="n">
+        <v>10</v>
+      </c>
+      <c r="B24" s="47" t="s">
+        <v>100</v>
+      </c>
+      <c r="C24" s="48" t="n">
+        <f aca="false">SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,$A24,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4,$A24+1,1))</f>
+        <v>0</v>
+      </c>
+      <c r="H24" s="47" t="str">
+        <f aca="false">IF(Settings!A27="","",Settings!A27)</f>
+        <v/>
+      </c>
+      <c r="I24" s="48" t="str">
+        <f aca="false">IF($H24="","",SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$B$6:$B$105,$H24,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,1,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4+1,1,1)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="46" t="n">
+        <v>11</v>
+      </c>
+      <c r="B25" s="47" t="s">
+        <v>101</v>
+      </c>
+      <c r="C25" s="48" t="n">
+        <f aca="false">SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,$A25,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4,$A25+1,1))</f>
+        <v>0</v>
+      </c>
+      <c r="H25" s="49" t="str">
+        <f aca="false">IF(Settings!A28="","",Settings!A28)</f>
+        <v/>
+      </c>
+      <c r="I25" s="50" t="str">
+        <f aca="false">IF($H25="","",SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$B$6:$B$105,$H25,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,1,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4+1,1,1)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="46" t="n">
+        <v>12</v>
+      </c>
+      <c r="B26" s="47" t="s">
+        <v>102</v>
+      </c>
+      <c r="C26" s="48" t="n">
+        <f aca="false">SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,$A26,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4,$A26+1,1))</f>
+        <v>0</v>
+      </c>
+      <c r="H26" s="49" t="str">
         <f aca="false">IF(Settings!A29="","",Settings!A29)</f>
         <v/>
       </c>
-      <c r="I23" s="47" t="str">
-        <f aca="false">IF($H23="","",SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$B$6:$B$105,$H23,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,1,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4+1,1,1)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H24" s="46" t="str">
+      <c r="I26" s="50" t="str">
+        <f aca="false">IF($H26="","",SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$B$6:$B$105,$H26,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,1,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4+1,1,1)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="H27" s="49" t="str">
         <f aca="false">IF(Settings!A30="","",Settings!A30)</f>
         <v/>
       </c>
-      <c r="I24" s="47" t="str">
-        <f aca="false">IF($H24="","",SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$B$6:$B$105,$H24,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,1,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4+1,1,1)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H25" s="46" t="str">
+      <c r="I27" s="50" t="str">
+        <f aca="false">IF($H27="","",SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$B$6:$B$105,$H27,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,1,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4+1,1,1)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B28" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="H28" s="49" t="str">
         <f aca="false">IF(Settings!A31="","",Settings!A31)</f>
         <v/>
       </c>
-      <c r="I25" s="47" t="str">
-        <f aca="false">IF($H25="","",SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$B$6:$B$105,$H25,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,1,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4+1,1,1)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H26" s="46" t="str">
+      <c r="I28" s="50" t="str">
+        <f aca="false">IF($H28="","",SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$B$6:$B$105,$H28,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,1,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4+1,1,1)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="B29" s="15" t="s">
+        <v>104</v>
+      </c>
+      <c r="C29" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="D29" s="15" t="s">
+        <v>105</v>
+      </c>
+      <c r="H29" s="49" t="str">
         <f aca="false">IF(Settings!A32="","",Settings!A32)</f>
         <v/>
       </c>
-      <c r="I26" s="47" t="str">
-        <f aca="false">IF($H26="","",SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$B$6:$B$105,$H26,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,1,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4+1,1,1)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H27" s="46" t="str">
+      <c r="I29" s="50" t="str">
+        <f aca="false">IF($H29="","",SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$B$6:$B$105,$H29,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,1,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4+1,1,1)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="46" t="n">
+        <v>1</v>
+      </c>
+      <c r="B30" s="47" t="s">
+        <v>106</v>
+      </c>
+      <c r="C30" s="48" t="n">
+        <f aca="false">SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,3*$A30-2,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4,3*$A30+1,1))</f>
+        <v>2970</v>
+      </c>
+      <c r="D30" s="48" t="n">
+        <f aca="false">SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$F$6:$F$105,"Paid",'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,3*$A30-2,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4,3*$A30+1,1))</f>
+        <v>2370</v>
+      </c>
+      <c r="H30" s="49" t="str">
         <f aca="false">IF(Settings!A33="","",Settings!A33)</f>
         <v/>
       </c>
-      <c r="I27" s="47" t="str">
-        <f aca="false">IF($H27="","",SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$B$6:$B$105,$H27,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,1,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4+1,1,1)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H28" s="46" t="str">
+      <c r="I30" s="50" t="str">
+        <f aca="false">IF($H30="","",SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$B$6:$B$105,$H30,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,1,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4+1,1,1)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="46" t="n">
+        <v>2</v>
+      </c>
+      <c r="B31" s="47" t="s">
+        <v>107</v>
+      </c>
+      <c r="C31" s="48" t="n">
+        <f aca="false">SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,3*$A31-2,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4,3*$A31+1,1))</f>
+        <v>0</v>
+      </c>
+      <c r="D31" s="48" t="n">
+        <f aca="false">SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$F$6:$F$105,"Paid",'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,3*$A31-2,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4,3*$A31+1,1))</f>
+        <v>0</v>
+      </c>
+      <c r="H31" s="49" t="str">
         <f aca="false">IF(Settings!A34="","",Settings!A34)</f>
         <v/>
       </c>
-      <c r="I28" s="47" t="str">
-        <f aca="false">IF($H28="","",SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$B$6:$B$105,$H28,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,1,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4+1,1,1)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H29" s="46" t="str">
+      <c r="I31" s="50" t="str">
+        <f aca="false">IF($H31="","",SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$B$6:$B$105,$H31,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,1,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4+1,1,1)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="46" t="n">
+        <v>3</v>
+      </c>
+      <c r="B32" s="47" t="s">
+        <v>108</v>
+      </c>
+      <c r="C32" s="48" t="n">
+        <f aca="false">SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,3*$A32-2,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4,3*$A32+1,1))</f>
+        <v>0</v>
+      </c>
+      <c r="D32" s="48" t="n">
+        <f aca="false">SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$F$6:$F$105,"Paid",'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,3*$A32-2,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4,3*$A32+1,1))</f>
+        <v>0</v>
+      </c>
+      <c r="H32" s="49" t="str">
         <f aca="false">IF(Settings!A35="","",Settings!A35)</f>
         <v/>
       </c>
-      <c r="I29" s="47" t="str">
-        <f aca="false">IF($H29="","",SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$B$6:$B$105,$H29,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,1,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4+1,1,1)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H30" s="46" t="str">
+      <c r="I32" s="50" t="str">
+        <f aca="false">IF($H32="","",SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$B$6:$B$105,$H32,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,1,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4+1,1,1)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="46" t="n">
+        <v>4</v>
+      </c>
+      <c r="B33" s="47" t="s">
+        <v>109</v>
+      </c>
+      <c r="C33" s="48" t="n">
+        <f aca="false">SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,3*$A33-2,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4,3*$A33+1,1))</f>
+        <v>0</v>
+      </c>
+      <c r="D33" s="48" t="n">
+        <f aca="false">SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$F$6:$F$105,"Paid",'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,3*$A33-2,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4,3*$A33+1,1))</f>
+        <v>0</v>
+      </c>
+      <c r="H33" s="49" t="str">
         <f aca="false">IF(Settings!A36="","",Settings!A36)</f>
         <v/>
       </c>
-      <c r="I30" s="47" t="str">
-        <f aca="false">IF($H30="","",SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$B$6:$B$105,$H30,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,1,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4+1,1,1)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H31" s="46" t="str">
+      <c r="I33" s="50" t="str">
+        <f aca="false">IF($H33="","",SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$B$6:$B$105,$H33,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,1,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4+1,1,1)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="H34" s="49" t="str">
         <f aca="false">IF(Settings!A37="","",Settings!A37)</f>
         <v/>
       </c>
-      <c r="I31" s="47" t="str">
-        <f aca="false">IF($H31="","",SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$B$6:$B$105,$H31,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,1,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4+1,1,1)))</f>
+      <c r="I34" s="50" t="str">
+        <f aca="false">IF($H34="","",SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$B$6:$B$105,$H34,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,1,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4+1,1,1)))</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="18">
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="B6:C6"/>
@@ -3721,10 +3883,18 @@
     <mergeCell ref="E7:F7"/>
     <mergeCell ref="H7:I7"/>
     <mergeCell ref="K7:L7"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="K9:L9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="K10:L10"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>

</xml_diff>

<commit_message>
Break-proof all products + Debt Payoff tab in budget template
Every sheet now carries password-free protection: formula cells are
locked against accidental edits while all input cells stay unlocked,
with a Start Here note explaining how to unprotect. Budget template
gains a Debt Payoff tab (8 tabs total): months-to-payoff and debt-free
date per debt via NPER, total interest, and an extra-payment tool
showing months and interest saved (avalanche method) — all values
verified against independently computed amortization math.

Listings updated: debt payoff in title/gallery/tags, break-proof
bullet on all three, new debt-payoff screenshot.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014AkUe8kkZr9XS2EdNVryQd
</commit_message>
<xml_diff>
--- a/products/freelance-invoice-income-tracker.xlsx
+++ b/products/freelance-invoice-income-tracker.xlsx
@@ -19,7 +19,7 @@
     <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Area" vbProcedure="false">'Income Log'!$A$1:$G$40</definedName>
     <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Area" vbProcedure="false">Invoice!$A$1:$D$35</definedName>
     <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">Settings!$A$1:$D$38</definedName>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">'Start Here'!$A$1:$H$26</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">'Start Here'!$A$1:$H$27</definedName>
     <definedName function="false" hidden="false" name="ClientList" vbProcedure="false">Settings!$A$18:$A$37</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="111">
   <si>
     <t xml:space="preserve">Freelance Invoice + Income Tracker</t>
   </si>
@@ -83,6 +83,9 @@
   </si>
   <si>
     <t xml:space="preserve">Works in Microsoft Excel (2016 or newer) and Google Sheets (upload to Drive, then Open with Google Sheets).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Formulas are protected so you can't break anything by accident — every cell meant for typing is unlocked. To change anything else: Review → Unprotect Sheet (no password).</t>
   </si>
   <si>
     <t xml:space="preserve">Settings</t>
@@ -743,17 +746,17 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+      <protection locked="false" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
@@ -775,13 +778,13 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+      <protection locked="false" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
@@ -791,9 +794,9 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+      <protection locked="false" hidden="false"/>
     </xf>
     <xf numFmtId="167" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
@@ -827,29 +830,29 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+      <protection locked="false" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="11" fillId="4" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
@@ -1207,11 +1210,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="94434206"/>
-        <c:axId val="95124837"/>
+        <c:axId val="25787640"/>
+        <c:axId val="94753621"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="94434206"/>
+        <c:axId val="25787640"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1243,7 +1246,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="95124837"/>
+        <c:crossAx val="94753621"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1251,7 +1254,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="95124837"/>
+        <c:axId val="94753621"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1293,7 +1296,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="94434206"/>
+        <c:crossAx val="25787640"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1534,10 +1537,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FF2E9E8F"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
@@ -1681,7 +1683,13 @@
         <v>16</v>
       </c>
     </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B26" s="9" t="s">
+        <v>17</v>
+      </c>
+    </row>
   </sheetData>
+  <sheetProtection sheet="true" formatCells="false" formatColumns="false" formatRows="false"/>
   <mergeCells count="7">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
@@ -1704,7 +1712,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FF1F3A5F"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:H37"/>
@@ -1720,7 +1727,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1732,7 +1739,7 @@
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1744,123 +1751,123 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B12" s="13" t="n">
         <v>0.085</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B14" s="11" t="n">
         <v>14</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D16" s="14" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="15" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C17" s="15" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1954,6 +1961,7 @@
       <c r="C37" s="11"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="true" formatCells="false" formatColumns="false" formatRows="false"/>
   <mergeCells count="2">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
@@ -1971,7 +1979,6 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FF1F3A5F"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:D34"/>
@@ -2011,7 +2018,7 @@
     </row>
     <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B5" s="18"/>
       <c r="C5" s="18"/>
@@ -2019,21 +2026,21 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="19" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D8" s="20" t="n">
         <v>46083</v>
@@ -2045,7 +2052,7 @@
         <v>billing@acmestudios.com</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D9" s="22" t="n">
         <f aca="false">IF($D$8="","",$D$8+Settings!$B$14)</f>
@@ -2060,21 +2067,21 @@
     </row>
     <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="15" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B13" s="11" t="n">
         <v>1</v>
@@ -2089,7 +2096,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B14" s="11" t="n">
         <v>2</v>
@@ -2194,7 +2201,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C26" s="25" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D26" s="26" t="n">
         <f aca="false">SUM(D13:D24)</f>
@@ -2213,7 +2220,7 @@
     </row>
     <row r="28" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C28" s="28" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D28" s="29" t="n">
         <f aca="false">D26+D27</f>
@@ -2222,7 +2229,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2236,13 +2243,14 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="31" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B34" s="31"/>
       <c r="C34" s="31"/>
       <c r="D34" s="31"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="true" formatCells="false" formatColumns="false" formatRows="false"/>
   <mergeCells count="6">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
@@ -2270,7 +2278,6 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FF1F3A5F"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:H105"/>
@@ -2288,7 +2295,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2300,7 +2307,7 @@
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2312,30 +2319,30 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G5" s="15" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2343,19 +2350,19 @@
         <v>46034</v>
       </c>
       <c r="B6" s="33" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C6" s="33" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D6" s="33" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E6" s="34" t="n">
         <v>1520</v>
       </c>
       <c r="F6" s="33" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G6" s="32" t="n">
         <v>46042</v>
@@ -2366,19 +2373,19 @@
         <v>46056</v>
       </c>
       <c r="B7" s="36" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C7" s="36" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D7" s="36" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E7" s="37" t="n">
         <v>850</v>
       </c>
       <c r="F7" s="36" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G7" s="35" t="n">
         <v>46068</v>
@@ -2389,19 +2396,19 @@
         <v>46083</v>
       </c>
       <c r="B8" s="33" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C8" s="33" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D8" s="33" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E8" s="34" t="n">
         <v>600</v>
       </c>
       <c r="F8" s="33" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G8" s="32"/>
     </row>
@@ -3279,6 +3286,7 @@
       <c r="G105" s="35"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="true" formatCells="false" formatColumns="false" formatRows="false" insertRows="false"/>
   <mergeCells count="2">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
@@ -3317,7 +3325,6 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FF2E9E8F"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:L34"/>
@@ -3336,7 +3343,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3352,7 +3359,7 @@
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -3368,7 +3375,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="7" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C4" s="11" t="n">
         <v>2026</v>
@@ -3376,19 +3383,19 @@
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="38" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C6" s="38"/>
       <c r="E6" s="38" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F6" s="38"/>
       <c r="H6" s="38" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="I6" s="38"/>
       <c r="K6" s="38" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="L6" s="38"/>
     </row>
@@ -3417,19 +3424,19 @@
     <row r="8" customFormat="false" ht="6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="38" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C9" s="38"/>
       <c r="E9" s="38" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F9" s="38"/>
       <c r="H9" s="38" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="I9" s="38"/>
       <c r="K9" s="38" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="L9" s="38"/>
     </row>
@@ -3457,27 +3464,27 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="5" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="15" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="H14" s="15" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="I14" s="15" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3485,7 +3492,7 @@
         <v>1</v>
       </c>
       <c r="B15" s="47" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C15" s="48" t="n">
         <f aca="false">SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,$A15,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4,$A15+1,1))</f>
@@ -3505,7 +3512,7 @@
         <v>2</v>
       </c>
       <c r="B16" s="47" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C16" s="48" t="n">
         <f aca="false">SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,$A16,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4,$A16+1,1))</f>
@@ -3525,7 +3532,7 @@
         <v>3</v>
       </c>
       <c r="B17" s="47" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C17" s="48" t="n">
         <f aca="false">SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,$A17,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4,$A17+1,1))</f>
@@ -3545,7 +3552,7 @@
         <v>4</v>
       </c>
       <c r="B18" s="47" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C18" s="48" t="n">
         <f aca="false">SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,$A18,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4,$A18+1,1))</f>
@@ -3565,7 +3572,7 @@
         <v>5</v>
       </c>
       <c r="B19" s="47" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C19" s="48" t="n">
         <f aca="false">SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,$A19,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4,$A19+1,1))</f>
@@ -3585,7 +3592,7 @@
         <v>6</v>
       </c>
       <c r="B20" s="47" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C20" s="48" t="n">
         <f aca="false">SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,$A20,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4,$A20+1,1))</f>
@@ -3605,7 +3612,7 @@
         <v>7</v>
       </c>
       <c r="B21" s="47" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C21" s="48" t="n">
         <f aca="false">SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,$A21,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4,$A21+1,1))</f>
@@ -3625,7 +3632,7 @@
         <v>8</v>
       </c>
       <c r="B22" s="47" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C22" s="48" t="n">
         <f aca="false">SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,$A22,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4,$A22+1,1))</f>
@@ -3645,7 +3652,7 @@
         <v>9</v>
       </c>
       <c r="B23" s="47" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C23" s="48" t="n">
         <f aca="false">SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,$A23,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4,$A23+1,1))</f>
@@ -3665,7 +3672,7 @@
         <v>10</v>
       </c>
       <c r="B24" s="47" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C24" s="48" t="n">
         <f aca="false">SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,$A24,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4,$A24+1,1))</f>
@@ -3685,7 +3692,7 @@
         <v>11</v>
       </c>
       <c r="B25" s="47" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C25" s="48" t="n">
         <f aca="false">SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,$A25,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4,$A25+1,1))</f>
@@ -3705,7 +3712,7 @@
         <v>12</v>
       </c>
       <c r="B26" s="47" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C26" s="48" t="n">
         <f aca="false">SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,$A26,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4,$A26+1,1))</f>
@@ -3732,7 +3739,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H28" s="49" t="str">
         <f aca="false">IF(Settings!A31="","",Settings!A31)</f>
@@ -3745,16 +3752,16 @@
     </row>
     <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="15" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B29" s="15" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C29" s="15" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D29" s="15" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H29" s="49" t="str">
         <f aca="false">IF(Settings!A32="","",Settings!A32)</f>
@@ -3770,7 +3777,7 @@
         <v>1</v>
       </c>
       <c r="B30" s="47" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C30" s="48" t="n">
         <f aca="false">SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,3*$A30-2,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4,3*$A30+1,1))</f>
@@ -3794,7 +3801,7 @@
         <v>2</v>
       </c>
       <c r="B31" s="47" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C31" s="48" t="n">
         <f aca="false">SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,3*$A31-2,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4,3*$A31+1,1))</f>
@@ -3818,7 +3825,7 @@
         <v>3</v>
       </c>
       <c r="B32" s="47" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C32" s="48" t="n">
         <f aca="false">SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,3*$A32-2,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4,3*$A32+1,1))</f>
@@ -3842,7 +3849,7 @@
         <v>4</v>
       </c>
       <c r="B33" s="47" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C33" s="48" t="n">
         <f aca="false">SUMIFS('Income Log'!$E$6:$E$105,'Income Log'!$A$6:$A$105,"&gt;="&amp;DATE($C$4,3*$A33-2,1),'Income Log'!$A$6:$A$105,"&lt;"&amp;DATE($C$4,3*$A33+1,1))</f>
@@ -3872,6 +3879,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection sheet="true" formatCells="false" formatColumns="false" formatRows="false"/>
   <mergeCells count="18">
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:L2"/>

</xml_diff>